<commit_message>
fig_1 and fig_2 SM,GEN
</commit_message>
<xml_diff>
--- a/data/2.0_balancing_selection/01_b2_candidates/Landrace_only_bal_description.xlsx
+++ b/data/2.0_balancing_selection/01_b2_candidates/Landrace_only_bal_description.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/subhashmahamkali/Downloads/1.miscellaneous/sorghum_project/B2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/subhashmahamkali/Documents/gwas_sap/data/2.0_balancing_selection/01_b2_candidates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92BAA99-EE68-4E48-82E7-CCEC8177388F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B56C6E94-C32F-2044-9BA6-5568500AEBFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="27040" windowHeight="15920" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="27040" windowHeight="15760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6324" uniqueCount="3160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6335" uniqueCount="3163">
   <si>
     <t>V1</t>
   </si>
@@ -9504,6 +9504,15 @@
   </si>
   <si>
     <t>Sobic.010G208800</t>
+  </si>
+  <si>
+    <t>dot_color</t>
+  </si>
+  <si>
+    <t>#1f78b4</t>
+  </si>
+  <si>
+    <t>#33a02c</t>
   </si>
 </sst>
 </file>
@@ -9553,33 +9562,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -79139,108 +79133,115 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E96EE8F1-6291-F14A-9DD2-CCBBBB08FBFF}">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>3160</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
         <v>53560029</v>
       </c>
-      <c r="C1">
+      <c r="C2" s="2">
         <v>53675012</v>
       </c>
-      <c r="D1">
+      <c r="D2" s="2">
         <v>2805.0559499999999</v>
       </c>
-      <c r="E1">
+      <c r="E2" s="2">
         <v>1</v>
       </c>
-      <c r="F1">
+      <c r="F2" s="2">
         <v>53635710</v>
       </c>
-      <c r="G1">
+      <c r="G2" s="2">
         <v>53640841</v>
       </c>
-      <c r="H1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J2" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
+      <c r="L2" s="2" t="s">
+        <v>3162</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
         <v>8</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B3" s="2">
         <v>14113586</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C3" s="2">
         <v>14312677</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D3" s="2">
         <v>3112.8637309999999</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E3" s="2">
         <v>8</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F3" s="2">
         <v>14274483</v>
       </c>
-      <c r="G2" s="2">
+      <c r="G3" s="2">
         <v>14283844</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>2709</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>2259</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2">
-        <v>62523232</v>
-      </c>
-      <c r="C3" s="2">
-        <v>62691998</v>
-      </c>
-      <c r="D3" s="2">
-        <v>3012.54315</v>
-      </c>
-      <c r="E3" s="2">
-        <v>6</v>
-      </c>
-      <c r="F3" s="2">
-        <v>62594307</v>
-      </c>
-      <c r="G3" s="2">
-        <v>62602526</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>2338</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>661</v>
-      </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L3" s="2" t="s">
+        <v>3162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>10</v>
       </c>
@@ -79271,11 +79272,11 @@
       <c r="J4" s="2" t="s">
         <v>3136</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-    </row>
+      <c r="L4" s="2" t="s">
+        <v>3161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>